<commit_message>
BITACORA T-007 Crear seed inicial de catalogos
</commit_message>
<xml_diff>
--- a/docs/BITACORA_presupuesto_costos_app_MVP_actualizada.xlsx
+++ b/docs/BITACORA_presupuesto_costos_app_MVP_actualizada.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROYECTOS PERSONALES\PRESUPUESTO_GASTOS\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79CF9537-A705-4C80-BD70-EB92589C1AC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE6A57AB-BC5B-410B-932A-51CD8851965B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16776" firstSheet="5" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7326,7 +7326,7 @@
       <c r="N10" s="6"/>
       <c r="O10" s="3"/>
       <c r="P10" s="1" t="s">
-        <v>406</v>
+        <v>671</v>
       </c>
       <c r="Q10" s="1"/>
     </row>
@@ -7367,7 +7367,7 @@
       <c r="N11" s="6"/>
       <c r="O11" s="3"/>
       <c r="P11" s="1" t="s">
-        <v>406</v>
+        <v>671</v>
       </c>
       <c r="Q11" s="1"/>
     </row>

</xml_diff>

<commit_message>
BITACORA SPRIT 1 CERRADO
</commit_message>
<xml_diff>
--- a/docs/BITACORA_presupuesto_costos_app_MVP_actualizada.xlsx
+++ b/docs/BITACORA_presupuesto_costos_app_MVP_actualizada.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROYECTOS PERSONALES\PRESUPUESTO_GASTOS\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE6A57AB-BC5B-410B-932A-51CD8851965B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C46EF75-9F75-4307-82F5-D73F3991B530}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16776" firstSheet="5" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7408,7 +7408,7 @@
       <c r="N12" s="6"/>
       <c r="O12" s="3"/>
       <c r="P12" s="1" t="s">
-        <v>406</v>
+        <v>671</v>
       </c>
       <c r="Q12" s="1"/>
     </row>
@@ -7449,7 +7449,7 @@
       <c r="N13" s="6"/>
       <c r="O13" s="3"/>
       <c r="P13" s="1" t="s">
-        <v>406</v>
+        <v>671</v>
       </c>
       <c r="Q13" s="1"/>
     </row>
@@ -7490,7 +7490,7 @@
       <c r="N14" s="6"/>
       <c r="O14" s="3"/>
       <c r="P14" s="1" t="s">
-        <v>406</v>
+        <v>671</v>
       </c>
       <c r="Q14" s="1"/>
     </row>
@@ -7531,7 +7531,7 @@
       <c r="N15" s="6"/>
       <c r="O15" s="3"/>
       <c r="P15" s="1" t="s">
-        <v>406</v>
+        <v>671</v>
       </c>
       <c r="Q15" s="1"/>
     </row>
@@ -7572,7 +7572,7 @@
       <c r="N16" s="6"/>
       <c r="O16" s="3"/>
       <c r="P16" s="1" t="s">
-        <v>406</v>
+        <v>671</v>
       </c>
       <c r="Q16" s="1"/>
     </row>
@@ -7613,7 +7613,7 @@
       <c r="N17" s="6"/>
       <c r="O17" s="3"/>
       <c r="P17" s="1" t="s">
-        <v>406</v>
+        <v>671</v>
       </c>
       <c r="Q17" s="1"/>
     </row>
@@ -7654,7 +7654,7 @@
       <c r="N18" s="6"/>
       <c r="O18" s="3"/>
       <c r="P18" s="1" t="s">
-        <v>406</v>
+        <v>671</v>
       </c>
       <c r="Q18" s="1"/>
     </row>

</xml_diff>

<commit_message>
BITACORA SPRINT 3 TERMINADO
</commit_message>
<xml_diff>
--- a/docs/BITACORA_presupuesto_costos_app_MVP_actualizada.xlsx
+++ b/docs/BITACORA_presupuesto_costos_app_MVP_actualizada.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROYECTOS PERSONALES\PRESUPUESTO_GASTOS\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A830D36E-84BD-41C9-A77E-3C61CA8987B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6E31041-D594-4C73-A6B8-0D7B05D4AFF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16776" firstSheet="5" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8105,7 +8105,7 @@
       <c r="N29" s="6"/>
       <c r="O29" s="3"/>
       <c r="P29" s="1" t="s">
-        <v>406</v>
+        <v>671</v>
       </c>
       <c r="Q29" s="1"/>
     </row>
@@ -8146,7 +8146,7 @@
       <c r="N30" s="6"/>
       <c r="O30" s="3"/>
       <c r="P30" s="1" t="s">
-        <v>406</v>
+        <v>671</v>
       </c>
       <c r="Q30" s="1"/>
     </row>
@@ -8187,7 +8187,7 @@
       <c r="N31" s="6"/>
       <c r="O31" s="3"/>
       <c r="P31" s="1" t="s">
-        <v>406</v>
+        <v>671</v>
       </c>
       <c r="Q31" s="1"/>
     </row>
@@ -8228,7 +8228,7 @@
       <c r="N32" s="6"/>
       <c r="O32" s="3"/>
       <c r="P32" s="1" t="s">
-        <v>406</v>
+        <v>671</v>
       </c>
       <c r="Q32" s="1"/>
     </row>
@@ -8269,7 +8269,7 @@
       <c r="N33" s="6"/>
       <c r="O33" s="3"/>
       <c r="P33" s="1" t="s">
-        <v>406</v>
+        <v>671</v>
       </c>
       <c r="Q33" s="1"/>
     </row>
@@ -8310,7 +8310,7 @@
       <c r="N34" s="6"/>
       <c r="O34" s="3"/>
       <c r="P34" s="1" t="s">
-        <v>406</v>
+        <v>671</v>
       </c>
       <c r="Q34" s="1"/>
     </row>

</xml_diff>